<commit_message>
Holders and IBANs: a bonifico between own accounts is a giroconto with one statement
New page Impostazioni → Titolari e IBAN: the holders' names and the full IBAN of
each account (also on the account form; IBAN check digits validated, never the
same IBAN on two accounts; new migration). On import, a bonifico naming a holder
(first/last name in any order) becomes a giroconto; naming the IBAN of another
account it gets both accounts straight away. The other statement imported later
joins that transfer instead of adding a second one. The two-bank sample uses
valid IBANs and the README says what to enter in the profile.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmHFHk7Z88SGFnopnWCqcC
</commit_message>
<xml_diff>
--- a/samples/dati_fittizi/due_banche/fineco_conto_risparmio_2022-01_2026-09.xlsx
+++ b/samples/dati_fittizi/due_banche/fineco_conto_risparmio_2022-01_2026-09.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - tredicesima</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - tredicesima</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Bonifico istantaneo a MARIO ROSSI IBAN IT60X0200801600000102345678 - anticipo acquisto casa</t>
+          <t>Bonifico istantaneo a MARIO ROSSI IBAN IT27X0200801600000102345678 - anticipo acquisto casa</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Bonifico istantaneo a MARIO ROSSI IBAN IT60X0200801600000102345678 - mobili casa nuova</t>
+          <t>Bonifico istantaneo a MARIO ROSSI IBAN IT27X0200801600000102345678 - mobili casa nuova</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - tredicesima</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - tredicesima</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - regali di nozze sul risparmio</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - regali di nozze sul risparmio</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -6366,7 +6366,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -6541,7 +6541,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Bonifico SEPA a MARIO ROSSI IBAN IT60X0200801600000102345678 - dentista</t>
+          <t>Bonifico SEPA a MARIO ROSSI IBAN IT27X0200801600000102345678 - dentista</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -7731,7 +7731,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -8256,7 +8256,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -9236,7 +9236,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Bonifico da MARIO ROSSI IBAN IT60X0200801600000102345678 - risparmio mensile</t>
+          <t>Bonifico da MARIO ROSSI IBAN IT27X0200801600000102345678 - risparmio mensile</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">

</xml_diff>